<commit_message>
Addition of production output files for ESC, PoHalf, RP2350, FPGA
</commit_message>
<xml_diff>
--- a/LilBoatBoards/MKII/PoHalf v2/Project Outputs for PoHalf/PoHalf.xlsx
+++ b/LilBoatBoards/MKII/PoHalf v2/Project Outputs for PoHalf/PoHalf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julmp\Documents\electric_boogaloo\LilBoatBoards\MKII\PoHalf v2\Project Outputs for PoHalf\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UWRT\Altium\electric_boogaloo\LilBoatBoards\MKII\PoHalf v2\Project Outputs for PoHalf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97903352-9F43-4F3A-B4C5-44B0F43A6D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{67CBE963-E14F-410A-88F5-46740281088A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11712" windowHeight="12960" xr2:uid="{6617505E-7342-47DE-87AB-8896E976A090}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{1C23F84E-D4D7-454E-B600-934555F6579A}"/>
   </bookViews>
   <sheets>
     <sheet name="PoHalf" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="274">
   <si>
     <t>Comment</t>
   </si>
@@ -59,18 +59,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Supplier Part Number 1</t>
-  </si>
-  <si>
-    <t>Supplier Part Number 2</t>
-  </si>
-  <si>
-    <t>Supplier Part Number 3</t>
-  </si>
-  <si>
-    <t>Supplier Part Number 4</t>
-  </si>
-  <si>
     <t>100uF electrolytic 35 V</t>
   </si>
   <si>
@@ -84,9 +72,6 @@
   </si>
   <si>
     <t>CAP ALUM 100UF 20% 35V SMD</t>
-  </si>
-  <si>
-    <t>667-EEE-1VA101XP</t>
   </si>
   <si>
     <t>100nF Ceramic 25V</t>
@@ -105,9 +90,6 @@
     <t>CAPACITOR_0.1uF_0402</t>
   </si>
   <si>
-    <t>478-7868-1-ND</t>
-  </si>
-  <si>
     <t>27pF Ceramic 50V</t>
   </si>
   <si>
@@ -121,9 +103,6 @@
     <t>CAPACITOR_0.000027uF_0402</t>
   </si>
   <si>
-    <t>445-5589-1-ND</t>
-  </si>
-  <si>
     <t>22uF electrolytic 35 V</t>
   </si>
   <si>
@@ -136,9 +115,6 @@
     <t>CAP ALUM 22UF 20% 35V SMD</t>
   </si>
   <si>
-    <t>PCE3952DKR-ND</t>
-  </si>
-  <si>
     <t>4700pF Ceramic 25V</t>
   </si>
   <si>
@@ -151,9 +127,6 @@
     <t>CAPACITOR_0.0047uF_0402</t>
   </si>
   <si>
-    <t>478-6195-1-ND</t>
-  </si>
-  <si>
     <t>CL05A104KA5NNNC</t>
   </si>
   <si>
@@ -164,9 +137,6 @@
   </si>
   <si>
     <t>CAP CER 0.1UF 25V X5R 0402</t>
-  </si>
-  <si>
-    <t>1276-1043-1-ND, CL05A104KA5NNNC</t>
   </si>
   <si>
     <t>100nF Ceramic 6.3V</t>
@@ -188,9 +158,6 @@
     <t>CAPACITOR_0.1uF_0603</t>
   </si>
   <si>
-    <t>399-15351-1-ND</t>
-  </si>
-  <si>
     <t>1uF Ceramic 16V</t>
   </si>
   <si>
@@ -204,9 +171,6 @@
     <t>CAPACITOR_1uF_0402</t>
   </si>
   <si>
-    <t>478-0402YD105KAT4ADKR-ND</t>
-  </si>
-  <si>
     <t>10uF Ceramic 25V</t>
   </si>
   <si>
@@ -223,9 +187,6 @@
     <t>CAPACITOR_10uF_1206</t>
   </si>
   <si>
-    <t>1276-1804-6-ND</t>
-  </si>
-  <si>
     <t>10uF Ceramic 6.3V</t>
   </si>
   <si>
@@ -239,9 +200,6 @@
     <t>CAPACITOR_10uF_0603</t>
   </si>
   <si>
-    <t>1276-1119-1-ND</t>
-  </si>
-  <si>
     <t>IN-S63AT5G</t>
   </si>
   <si>
@@ -258,9 +216,6 @@
     <t>LED_Green_0603_3V</t>
   </si>
   <si>
-    <t>1830-1062-1-ND</t>
-  </si>
-  <si>
     <t>EAST1616RGBB4</t>
   </si>
   <si>
@@ -274,9 +229,6 @@
   </si>
   <si>
     <t>LED_RGB_4SMD</t>
-  </si>
-  <si>
-    <t>1080-1552-1-ND</t>
   </si>
   <si>
     <t>150060BS75000</t>
@@ -292,9 +244,6 @@
     <t>LED_Blue_0603</t>
   </si>
   <si>
-    <t>732-4966-1-ND</t>
-  </si>
-  <si>
     <t>0685H9150-01</t>
   </si>
   <si>
@@ -341,9 +290,6 @@
     <t>CONN_MOLEX_MICROFIT+_6POS_R/A</t>
   </si>
   <si>
-    <t>900-2125280600-ND</t>
-  </si>
-  <si>
     <t>Molex Microfit+ _x000D_
 212528 4 POS R/A Black</t>
   </si>
@@ -357,9 +303,6 @@
     <t>CONN_MOLEX_MICROFIT+_4POS_R/A</t>
   </si>
   <si>
-    <t>900-2125280400-ND</t>
-  </si>
-  <si>
     <t>Mini-Fit Jr R/A</t>
   </si>
   <si>
@@ -376,9 +319,6 @@
     <t>CONN_MOLEX_MINIFIT JR_4POS_R/A</t>
   </si>
   <si>
-    <t>WM13112-ND</t>
-  </si>
-  <si>
     <t>JST GH VERT</t>
   </si>
   <si>
@@ -392,9 +332,6 @@
   </si>
   <si>
     <t>CONN_JST_GH_4POS_VERT</t>
-  </si>
-  <si>
-    <t>455-1580-1-ND</t>
   </si>
   <si>
     <t>PP45 R/A</t>
@@ -413,18 +350,6 @@
     <t>CONN_ANDERSON_2x2_R/A</t>
   </si>
   <si>
-    <t>2243-1337G1-ND</t>
-  </si>
-  <si>
-    <t>2243-1336G1-ND</t>
-  </si>
-  <si>
-    <t>2243-1327-BK-ND</t>
-  </si>
-  <si>
-    <t>A102007-ND</t>
-  </si>
-  <si>
     <t>Redcube M4 Term 85A</t>
   </si>
   <si>
@@ -450,9 +375,6 @@
     <t>CONN_MICROUSB</t>
   </si>
   <si>
-    <t>609-4613-1-ND</t>
-  </si>
-  <si>
     <t>61300311121</t>
   </si>
   <si>
@@ -475,9 +397,6 @@
   </si>
   <si>
     <t>CONN_JST_GH_2POS_VERT</t>
-  </si>
-  <si>
-    <t>455-1564-1-ND</t>
   </si>
   <si>
     <t>Molex Minifit Jr. 5569 _x000D_
@@ -493,9 +412,6 @@
     <t>CONN_MOLEX_MINIFIT JR_2POS_R/A</t>
   </si>
   <si>
-    <t>WM1351-ND</t>
-  </si>
-  <si>
     <t>XH2.54 VERT</t>
   </si>
   <si>
@@ -532,9 +448,6 @@
     <t>MOSFET_7DP-T1-GE3_VIS</t>
   </si>
   <si>
-    <t>78-SIR167DP-T1-GE3</t>
-  </si>
-  <si>
     <t>MMBT3904-7-F</t>
   </si>
   <si>
@@ -562,9 +475,6 @@
     <t>SOT-23-3</t>
   </si>
   <si>
-    <t>785-1004-1-ND</t>
-  </si>
-  <si>
     <t>MOSFET N-CH 30V 5.8A SOT-23-3</t>
   </si>
   <si>
@@ -583,9 +493,6 @@
     <t>MMBT2907A-7-F</t>
   </si>
   <si>
-    <t>MMBT2907A-FDICT-ND</t>
-  </si>
-  <si>
     <t>4.7k Ohm 5% 1/10W</t>
   </si>
   <si>
@@ -601,9 +508,6 @@
     <t>RESISTOR_4.7K_0603</t>
   </si>
   <si>
-    <t>RMCF0603JT4K70CT-ND</t>
-  </si>
-  <si>
     <t>10k Ohm 1% 1/16W</t>
   </si>
   <si>
@@ -619,9 +523,6 @@
     <t>RESISTOR_10K_0402</t>
   </si>
   <si>
-    <t>YAG3436CT-ND</t>
-  </si>
-  <si>
     <t>1k Ohm 1% 1/16W</t>
   </si>
   <si>
@@ -634,9 +535,6 @@
     <t>RESISTOR_1K_0402</t>
   </si>
   <si>
-    <t>13-AC0402FR-131KLCT-ND</t>
-  </si>
-  <si>
     <t>1k Ohm 5% 1/8W</t>
   </si>
   <si>
@@ -649,9 +547,6 @@
     <t>RESISTOR_1K_0603</t>
   </si>
   <si>
-    <t>2019-RK73B1JTTD102JCT-ND</t>
-  </si>
-  <si>
     <t>60.4 Ohm 1% 1/16W</t>
   </si>
   <si>
@@ -664,9 +559,6 @@
     <t>RESISTOR_60.4_0402</t>
   </si>
   <si>
-    <t>13-AC0402FR-0760R4LCT-ND</t>
-  </si>
-  <si>
     <t>27 Ohm 1% 1/16W</t>
   </si>
   <si>
@@ -679,9 +571,6 @@
     <t>RESISTOR_27_0402</t>
   </si>
   <si>
-    <t>YAG5278DKR-ND</t>
-  </si>
-  <si>
     <t>10k Ohm 5% 1/10W</t>
   </si>
   <si>
@@ -694,9 +583,6 @@
     <t>RESISTOR_10K_0603</t>
   </si>
   <si>
-    <t>2019-RK73B1JTTD103JCT-ND</t>
-  </si>
-  <si>
     <t>604 Ohm 1% 1/16W</t>
   </si>
   <si>
@@ -709,9 +595,6 @@
     <t>RESISTOR_604_0402</t>
   </si>
   <si>
-    <t>13-AC0402FR-07604RLCT-ND</t>
-  </si>
-  <si>
     <t>3.9k Ohm 5% 1/10W</t>
   </si>
   <si>
@@ -724,9 +607,6 @@
     <t>RESISTOR_3.9K_0603</t>
   </si>
   <si>
-    <t>P3.90KHCT-ND</t>
-  </si>
-  <si>
     <t>200 Ohm 1% 1/16W</t>
   </si>
   <si>
@@ -739,9 +619,6 @@
     <t>RESISTOR_200_0402</t>
   </si>
   <si>
-    <t>YAG3453CT-ND</t>
-  </si>
-  <si>
     <t>10k Ohm 0.5% 1/10W</t>
   </si>
   <si>
@@ -754,9 +631,6 @@
     <t>RESISTOR_10K_0.5%_0603</t>
   </si>
   <si>
-    <t>749-1695-1-ND</t>
-  </si>
-  <si>
     <t>1k Ohm 5% 1/10W</t>
   </si>
   <si>
@@ -769,9 +643,6 @@
     <t>RESISTOR_1K_0.5%_0603</t>
   </si>
   <si>
-    <t>749-1693-1-ND</t>
-  </si>
-  <si>
     <t>100k Ohm 0.5% 1/10W</t>
   </si>
   <si>
@@ -784,9 +655,6 @@
     <t>RESISTOR_100K_0.5%_0603</t>
   </si>
   <si>
-    <t>311-2395-1-ND</t>
-  </si>
-  <si>
     <t>47K</t>
   </si>
   <si>
@@ -799,9 +667,6 @@
     <t>RC0603JR-1347KL</t>
   </si>
   <si>
-    <t>667-ERJ-3GEYJ473V</t>
-  </si>
-  <si>
     <t>20k Ohm 1% 1/16W</t>
   </si>
   <si>
@@ -814,9 +679,6 @@
     <t>RESISTOR_20K_0402</t>
   </si>
   <si>
-    <t>YAG3454CT-ND</t>
-  </si>
-  <si>
     <t>RES 8.56K OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -829,9 +691,6 @@
     <t>RESISTOR_8.56K_1%_0402</t>
   </si>
   <si>
-    <t>2019-RN73H1ETTP8561F50CT-ND</t>
-  </si>
-  <si>
     <t>RT0402BRD071K82L</t>
   </si>
   <si>
@@ -862,9 +721,6 @@
     <t>CAS-220TA_CAN_TERM</t>
   </si>
   <si>
-    <t>CAS220JCT-ND</t>
-  </si>
-  <si>
     <t>434123025826</t>
   </si>
   <si>
@@ -928,9 +784,6 @@
     <t>SOIC127P600X175-14N</t>
   </si>
   <si>
-    <t>MCP3428-E/SL-ND</t>
-  </si>
-  <si>
     <t>CAN Transceiver</t>
   </si>
   <si>
@@ -946,9 +799,6 @@
     <t>TJA1442AT</t>
   </si>
   <si>
-    <t>771-TJA1442AT/0Z</t>
-  </si>
-  <si>
     <t>W25Q128JVSIQ</t>
   </si>
   <si>
@@ -961,9 +811,6 @@
     <t>SOIC-8 W25QxJV</t>
   </si>
   <si>
-    <t>W25Q128JVSIQ-ND</t>
-  </si>
-  <si>
     <t>SHT14 SENSOR HUMID/TEMP</t>
   </si>
   <si>
@@ -979,9 +826,6 @@
     <t>SHT41-AD1B-R2</t>
   </si>
   <si>
-    <t>1649-SHT41-AD1B-R2CT-ND</t>
-  </si>
-  <si>
     <t>TC4432EOA713</t>
   </si>
   <si>
@@ -994,9 +838,6 @@
     <t>SOIC8-N_MC_MCH</t>
   </si>
   <si>
-    <t>TC4432EOA713CT-ND</t>
-  </si>
-  <si>
     <t>DG448DV-T1-E3</t>
   </si>
   <si>
@@ -1009,9 +850,6 @@
     <t>TSOP6_DG_VIS-M</t>
   </si>
   <si>
-    <t>781-DG448DV-E3</t>
-  </si>
-  <si>
     <t>LM1117IMPX-3.3/NOPB</t>
   </si>
   <si>
@@ -1037,9 +875,6 @@
   </si>
   <si>
     <t>CRYSTAL_12MHz_SMD_SMALL</t>
-  </si>
-  <si>
-    <t>2151-RH100-12.000-18-2030-EXT-TRCT-ND</t>
   </si>
 </sst>
 </file>
@@ -1438,15 +1273,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C00E92-6D74-4A11-AEB9-EB6A97D6DA76}">
-  <dimension ref="A1:J64"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96A7D9F5-ACC6-45A3-956F-035829E23D0A}">
+  <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="6" width="19" customWidth="1"/>
-    <col min="7" max="10" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1465,1636 +1299,1266 @@
       <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="F2" s="1">
         <v>2</v>
       </c>
-      <c r="G2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="F3" s="1">
         <v>3</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="F4" s="1">
         <v>2</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F5" s="1">
         <v>2</v>
       </c>
-      <c r="G5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="F7" s="1">
         <v>2</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F8" s="1">
         <v>9</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="F9" s="1">
         <v>2</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="F10" s="1">
         <v>3</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="F11" s="1">
         <v>1</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="F12" s="1">
         <v>2</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="F13" s="1">
         <v>6</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F14" s="1">
         <v>1</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-    </row>
-    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F15" s="1">
-        <v>1</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="F16" s="1">
         <v>3</v>
       </c>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="F17" s="1">
         <v>1</v>
       </c>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-    </row>
-    <row r="18" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="F18" s="1">
         <v>2</v>
       </c>
-      <c r="G18" s="2" t="s">
+    </row>
+    <row r="19" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-    </row>
-    <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B19" s="3" t="s">
+      <c r="E22" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="F22" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F19" s="1">
-        <v>1</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-    </row>
-    <row r="20" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F20" s="1">
-        <v>1</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="F21" s="1">
-        <v>1</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-    </row>
-    <row r="22" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F22" s="1">
-        <v>1</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>126</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="F23" s="1">
         <v>4</v>
       </c>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-    </row>
-    <row r="24" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>127</v>
+        <v>102</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>131</v>
+        <v>106</v>
       </c>
       <c r="F24" s="1">
         <v>1</v>
       </c>
-      <c r="G24" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>135</v>
+        <v>109</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>136</v>
+        <v>110</v>
       </c>
       <c r="F25" s="1">
         <v>1</v>
       </c>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>138</v>
+        <v>112</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>139</v>
+        <v>113</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>140</v>
+        <v>114</v>
       </c>
       <c r="F26" s="1">
         <v>1</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-    </row>
-    <row r="27" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>142</v>
+        <v>115</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="F27" s="1">
         <v>1</v>
       </c>
-      <c r="G27" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
       <c r="F28" s="1">
         <v>2</v>
       </c>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="F29" s="1">
         <v>2</v>
       </c>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>156</v>
+        <v>128</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>157</v>
+        <v>129</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
       <c r="F30" s="1">
         <v>3</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>160</v>
+        <v>131</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>161</v>
+        <v>132</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>162</v>
+        <v>133</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>163</v>
+        <v>134</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="F31" s="1">
         <v>2</v>
       </c>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>167</v>
+        <v>138</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>168</v>
+        <v>139</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="F32" s="1">
         <v>1</v>
       </c>
-      <c r="G32" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>168</v>
+        <v>139</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="F33" s="1">
         <v>1</v>
       </c>
-      <c r="G33" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>173</v>
+        <v>143</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>174</v>
+        <v>144</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>168</v>
+        <v>139</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="F34" s="1">
         <v>1</v>
       </c>
-      <c r="G34" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>177</v>
+        <v>146</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>178</v>
+        <v>147</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>179</v>
+        <v>148</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>181</v>
+        <v>150</v>
       </c>
       <c r="F35" s="1">
         <v>4</v>
       </c>
-      <c r="G35" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>183</v>
+        <v>151</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>187</v>
+        <v>155</v>
       </c>
       <c r="F36" s="1">
         <v>5</v>
       </c>
-      <c r="G36" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>189</v>
+        <v>156</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>190</v>
+        <v>157</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>191</v>
+        <v>158</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>192</v>
+        <v>159</v>
       </c>
       <c r="F37" s="1">
         <v>4</v>
       </c>
-      <c r="G37" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="1"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>194</v>
+        <v>160</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>195</v>
+        <v>161</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>196</v>
+        <v>162</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>197</v>
+        <v>163</v>
       </c>
       <c r="F38" s="1">
         <v>8</v>
       </c>
-      <c r="G38" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>199</v>
+        <v>164</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>200</v>
+        <v>165</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>201</v>
+        <v>166</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="F39" s="1">
         <v>2</v>
       </c>
-      <c r="G39" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="H39" s="1"/>
-      <c r="I39" s="1"/>
-      <c r="J39" s="1"/>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>204</v>
+        <v>168</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>205</v>
+        <v>169</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>207</v>
+        <v>171</v>
       </c>
       <c r="F40" s="1">
         <v>2</v>
       </c>
-      <c r="G40" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>209</v>
+        <v>172</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>210</v>
+        <v>173</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>211</v>
+        <v>174</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>212</v>
+        <v>175</v>
       </c>
       <c r="F41" s="1">
         <v>3</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>214</v>
+        <v>176</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>215</v>
+        <v>177</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>216</v>
+        <v>178</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>217</v>
+        <v>179</v>
       </c>
       <c r="F42" s="1">
         <v>1</v>
       </c>
-      <c r="G42" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>219</v>
+        <v>180</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>220</v>
+        <v>181</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>221</v>
+        <v>182</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>222</v>
+        <v>183</v>
       </c>
       <c r="F43" s="1">
         <v>4</v>
       </c>
-      <c r="G43" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="H43" s="1"/>
-      <c r="I43" s="1"/>
-      <c r="J43" s="1"/>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>224</v>
+        <v>184</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>225</v>
+        <v>185</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>226</v>
+        <v>186</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>227</v>
+        <v>187</v>
       </c>
       <c r="F44" s="1">
         <v>2</v>
       </c>
-      <c r="G44" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-      <c r="J44" s="1"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>229</v>
+        <v>188</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
       <c r="F45" s="1">
         <v>5</v>
       </c>
-      <c r="G45" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="H45" s="1"/>
-      <c r="I45" s="1"/>
-      <c r="J45" s="1"/>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>234</v>
+        <v>192</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>235</v>
+        <v>193</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>236</v>
+        <v>194</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>237</v>
+        <v>195</v>
       </c>
       <c r="F46" s="1">
         <v>3</v>
       </c>
-      <c r="G46" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-      <c r="J46" s="1"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>239</v>
+        <v>196</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>240</v>
+        <v>197</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>241</v>
+        <v>198</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>180</v>
+        <v>149</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>242</v>
+        <v>199</v>
       </c>
       <c r="F47" s="1">
         <v>2</v>
       </c>
-      <c r="G47" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-      <c r="J47" s="1"/>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>244</v>
+        <v>200</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>245</v>
+        <v>201</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>246</v>
+        <v>202</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>247</v>
+        <v>203</v>
       </c>
       <c r="F48" s="1">
         <v>1</v>
       </c>
-      <c r="G48" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>249</v>
+        <v>204</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>250</v>
+        <v>205</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>251</v>
+        <v>206</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>252</v>
+        <v>207</v>
       </c>
       <c r="F49" s="1">
         <v>1</v>
       </c>
-      <c r="G49" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-      <c r="J49" s="1"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>254</v>
+        <v>208</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>255</v>
+        <v>209</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>257</v>
+        <v>211</v>
       </c>
       <c r="F50" s="1">
         <v>1</v>
       </c>
-      <c r="G50" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-      <c r="J50" s="1"/>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>259</v>
+        <v>212</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>260</v>
+        <v>213</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>261</v>
+        <v>214</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>262</v>
+        <v>215</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>263</v>
+        <v>216</v>
       </c>
       <c r="F51" s="1">
         <v>1</v>
       </c>
-      <c r="G51" s="1"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-      <c r="J51" s="1"/>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>264</v>
+        <v>217</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>265</v>
+        <v>218</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>266</v>
+        <v>219</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>267</v>
+        <v>220</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>268</v>
+        <v>221</v>
       </c>
       <c r="F52" s="1">
         <v>1</v>
       </c>
-      <c r="G52" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="H52" s="1"/>
-      <c r="I52" s="1"/>
-      <c r="J52" s="1"/>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>270</v>
+        <v>222</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>271</v>
+        <v>223</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>272</v>
+        <v>224</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>273</v>
+        <v>225</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>274</v>
+        <v>226</v>
       </c>
       <c r="F53" s="1">
         <v>2</v>
       </c>
-      <c r="G53" s="1"/>
-      <c r="H53" s="1"/>
-      <c r="I53" s="1"/>
-      <c r="J53" s="1"/>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>275</v>
+        <v>227</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>276</v>
+        <v>228</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>277</v>
+        <v>229</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>278</v>
+        <v>230</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>275</v>
+        <v>227</v>
       </c>
       <c r="F54" s="1">
         <v>1</v>
       </c>
-      <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
-      <c r="I54" s="1"/>
-      <c r="J54" s="1"/>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>279</v>
+        <v>231</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>280</v>
+        <v>232</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>281</v>
+        <v>233</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>282</v>
+        <v>234</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>279</v>
+        <v>231</v>
       </c>
       <c r="F55" s="1">
         <v>1</v>
       </c>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
-      <c r="I55" s="1"/>
-      <c r="J55" s="1"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>283</v>
+        <v>235</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>284</v>
+        <v>236</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>285</v>
+        <v>237</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>286</v>
+        <v>238</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>283</v>
+        <v>235</v>
       </c>
       <c r="F56" s="1">
         <v>1</v>
       </c>
-      <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
-      <c r="I56" s="1"/>
-      <c r="J56" s="1"/>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>287</v>
+        <v>239</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>288</v>
+        <v>240</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>289</v>
+        <v>241</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>290</v>
+        <v>242</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>287</v>
+        <v>239</v>
       </c>
       <c r="F57" s="1">
         <v>1</v>
       </c>
-      <c r="G57" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="H57" s="1"/>
-      <c r="I57" s="1"/>
-      <c r="J57" s="1"/>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>292</v>
+        <v>243</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>293</v>
+        <v>244</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>294</v>
+        <v>245</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>295</v>
+        <v>246</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>296</v>
+        <v>247</v>
       </c>
       <c r="F58" s="1">
         <v>1</v>
       </c>
-      <c r="G58" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="H58" s="1"/>
-      <c r="I58" s="1"/>
-      <c r="J58" s="1"/>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>298</v>
+        <v>248</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>299</v>
+        <v>249</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>301</v>
+        <v>251</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>298</v>
+        <v>248</v>
       </c>
       <c r="F59" s="1">
         <v>1</v>
       </c>
-      <c r="G59" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H59" s="1"/>
-      <c r="I59" s="1"/>
-      <c r="J59" s="1"/>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>303</v>
+        <v>252</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>304</v>
+        <v>253</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>305</v>
+        <v>254</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>306</v>
+        <v>255</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>307</v>
+        <v>256</v>
       </c>
       <c r="F60" s="1">
         <v>1</v>
       </c>
-      <c r="G60" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="H60" s="1"/>
-      <c r="I60" s="1"/>
-      <c r="J60" s="1"/>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>309</v>
+        <v>257</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>310</v>
+        <v>258</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>311</v>
+        <v>259</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>312</v>
+        <v>260</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>309</v>
+        <v>257</v>
       </c>
       <c r="F61" s="1">
         <v>2</v>
       </c>
-      <c r="G61" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="H61" s="1"/>
-      <c r="I61" s="1"/>
-      <c r="J61" s="1"/>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>314</v>
+        <v>261</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>315</v>
+        <v>262</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>316</v>
+        <v>263</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>317</v>
+        <v>264</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>314</v>
+        <v>261</v>
       </c>
       <c r="F62" s="1">
         <v>1</v>
       </c>
-      <c r="G62" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="H62" s="1"/>
-      <c r="I62" s="1"/>
-      <c r="J62" s="1"/>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>319</v>
+        <v>265</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>320</v>
+        <v>266</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>321</v>
+        <v>267</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>322</v>
+        <v>268</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>319</v>
+        <v>265</v>
       </c>
       <c r="F63" s="1">
         <v>1</v>
       </c>
-      <c r="G63" s="1"/>
-      <c r="H63" s="1"/>
-      <c r="I63" s="1"/>
-      <c r="J63" s="1"/>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>323</v>
+        <v>269</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>324</v>
+        <v>270</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>325</v>
+        <v>271</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>326</v>
+        <v>272</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>327</v>
+        <v>273</v>
       </c>
       <c r="F64" s="1">
         <v>1</v>
       </c>
-      <c r="G64" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="H64" s="1"/>
-      <c r="I64" s="1"/>
-      <c r="J64" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>